<commit_message>
Revise KP: NIC 1143, 49× 4MBIR-28-TMLW, PTZ 2BPBDD-4794-20 with ST-1
Replace the unidentified 4BHNN0 cameras with the requested models, require ST-1 on all cameras, pick the cheapest RUWARE PTZ that has ST-1, and regenerate Word and Excel quotes (revision 2).

Co-authored-by: Yury1331 <Yury1331@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kp/2026-08-14-neurostation-4bhnn0/КП_поставка_NeuroStation_Astra_9800R_4BHNN0.xlsx
+++ b/kp/2026-08-14-neurostation-4bhnn0/КП_поставка_NeuroStation_Astra_9800R_4BHNN0.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="КП" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Источники цен" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="КП" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники цен" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'КП'!$A$12:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'КП'!$A$12:$I$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'КП'!$1:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'КП'!$A$1:$I$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'КП'!$A$1:$I$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -751,7 +751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -783,7 +783,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>№ КП-2026-08-14-001 от 14.08.2026  ·  Поставка видеорегистраторов TRASSIR и цифровых камер  ·  Цены с НДС 22%, ориентир открытого рынка, не оферта</t>
+          <t>№ КП-2026-08-14-001 ред. 2 от 14.08.2026  ·  2× NVR TRASSIR + 1× НИЦ 1143 + 49× 4MBIR-28-TMLW + 1× PTZ  ·  все камеры со СТ-1  ·  цены с НДС 22%</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
@@ -830,7 +830,7 @@
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>к заполнению (ориентир: дилеры TRASSIR / DSSL, НИЦ «Технологии»)</t>
+          <t>к заполнению (DSSL / TRASSIR, НИЦ «Технологии», ООО «Айпи Плюс» / РУВЕР)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>NVR: 5–15 раб. дней при наличии; камеры НИЦ — под заказ</t>
+          <t>NVR: 5–15 раб. дней при наличии; камеры НИЦ и РУВЕР — под заказ</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>IP-видеорегистратор TRASSIR NeuroStation Astra 9800R/128-S, 128 каналов, Astra Linux SE «Смоленск», 8×HDD 3.5" (диски не входят), 2 лицензии Neuro Detector в комплекте</t>
+          <t>IP-видеорегистратор TRASSIR NeuroStation Astra 9800R/128-S, 128 каналов, Astra Linux SE «Смоленск», 8×HDD 3.5" (диски не входят), 2 лицензии Neuro Detector в комплекте. СТ-1 / реестры ПП №719 и №878</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -978,12 +978,12 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Камера видеонаблюдения цифровая 4 Мп, прошивка Nexus. Артикул 4BHNN0-0-0-0 (производитель/корпус/объектив — подтвердить у НИЦ)</t>
+          <t>Купольная IP-камера 4 Мп НИЦ модель 1143, мотор 2.7–13.5 мм, ИК до 35 м, IP66/IK10, ПО Nexus. Производство РФ, СТ-1 на партию</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>4BHNN0-0-0-0</t>
+          <t>4MP-DOM-2.7-13.5M Nexus</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
@@ -992,632 +992,698 @@
         </is>
       </c>
       <c r="E14" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>23800</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>23800</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>4291.8</v>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>Спецификация НИЦ PDF; ориентир цены 4MP-DOM-2.7-13.5M; СТ-1 запросить на партию</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Уличная цилиндрическая IP-камера 4 Мп Mini Bullet, объектив 2.8 мм, ИК + белый свет, микрофон. Производитель РУВЕР, СТ-1</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>4MBIR-28-TMLW</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>18500</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>906500</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>163467.21</v>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>https://www.ipplus.ru/catalog/ip-kamery/ip-kamery-4mp/4mbir-28-tmlw ; st_1=true</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>PTZ уличная 2 Мп, зум ×20 (4.7–94 мм), IP66. Самая недорогая PTZ РУВЕР/Айпи Плюс с СТ-1 в серии 2 Мп (×10 без СТ-1 не предлагаются)</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>2BPBDD-4794-20</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>92750</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>92750</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>16725.41</v>
+      </c>
+      <c r="I16" s="14" t="inlineStr">
+        <is>
+          <t>https://www.ipplus.ru/catalog/ptz-kamery/ptz-kamery-2mp/2bpbdd-4794-20 ; реестр Минпромторга</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Итого по запросу (позиции 1–4), камеры 51 шт. со СТ-1</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="n"/>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="17" t="n"/>
+      <c r="G17" s="18" t="n">
+        <v>1978530</v>
+      </c>
+      <c r="H17" s="18" t="n">
+        <v>356784.1</v>
+      </c>
+      <c r="I17" s="19" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>2. Обязательно к поставке для работоспособности (в регистраторе нет лицензий на IP-камеры; камеры НИЦ/РУВЕР не native TRASSIR)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Наименование</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Цена с НДС, ₽</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Сумма с НДС, ₽</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>в т.ч. НДС 22%, ₽</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Лицензия TRASSIR AnyIP (TRASSIR OS) — подключение 1 IP-камеры любого производителя</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>DSSL 57885</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="F14" s="15" t="n">
-        <v>22000</v>
-      </c>
-      <c r="G14" s="15" t="n">
-        <v>1122000</v>
-      </c>
-      <c r="H14" s="15" t="n">
-        <v>202327.87</v>
-      </c>
-      <c r="I14" s="14" t="inlineStr">
-        <is>
-          <t>Ориентир опта НИЦ 4 Мп: 15–25 тыс. ₽; цена подлежит подтверждению</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Итого по запросу (позиции 1–2)</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
-      <c r="G15" s="18" t="n">
-        <v>2077480</v>
-      </c>
-      <c r="H15" s="18" t="n">
-        <v>374627.54</v>
-      </c>
-      <c r="I15" s="19" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>2. Обязательно к поставке для работоспособности (в регистраторе нет лицензий на IP-камеры; камеры не native TRASSIR)</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="F21" s="22" t="n">
+        <v>5090</v>
+      </c>
+      <c r="G21" s="22" t="n">
+        <v>259590</v>
+      </c>
+      <c r="H21" s="22" t="n">
+        <v>46811.31</v>
+      </c>
+      <c r="I21" s="21" t="inlineStr">
+        <is>
+          <t>Цена DSSL с 01.04.2026; без лицензии камера к NVR не подключается</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>Итого работоспособный минимум (позиции 1–5)</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="n"/>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24" t="n"/>
+      <c r="F22" s="24" t="n"/>
+      <c r="G22" s="25" t="n">
+        <v>2238120</v>
+      </c>
+      <c r="H22" s="25" t="n">
+        <v>403595.41</v>
+      </c>
+      <c r="I22" s="26" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>3. Рекомендуемые опции (в исходном запросе отсутствуют)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>Артикул</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Цена с НДС, ₽</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>Сумма с НДС, ₽</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t>в т.ч. НДС 22%, ₽</t>
         </is>
       </c>
-      <c r="I18" s="9" t="inlineStr">
+      <c r="I25" s="9" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="B19" s="21" t="inlineStr">
-        <is>
-          <t>Лицензия TRASSIR AnyIP (TRASSIR OS) — подключение 1 IP-камеры любого производителя</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>DSSL 57885</t>
-        </is>
-      </c>
-      <c r="D19" s="20" t="inlineStr">
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>HDD 10 ТБ Seagate SkyHawk AI, 3.5" SATA, рекомендован DSSL для NeuroStation 8-disk</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>ST10000VE001</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
         <is>
           <t>шт.</t>
         </is>
       </c>
-      <c r="E19" s="20" t="n">
-        <v>51</v>
-      </c>
-      <c r="F19" s="22" t="n">
-        <v>5090</v>
-      </c>
-      <c r="G19" s="22" t="n">
-        <v>259590</v>
-      </c>
-      <c r="H19" s="22" t="n">
-        <v>46811.31</v>
-      </c>
-      <c r="I19" s="21" t="inlineStr">
-        <is>
-          <t>Цена DSSL с 01.04.2026; без лицензии камера к NVR не подключается</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="23" t="inlineStr">
-        <is>
-          <t>Итого работоспособный минимум (позиции 1–3)</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="25" t="n">
-        <v>2337070</v>
-      </c>
-      <c r="H20" s="25" t="n">
-        <v>421438.85</v>
-      </c>
-      <c r="I20" s="26" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>3. Рекомендуемые опции (в исходном запросе отсутствуют)</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Наименование</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Артикул</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Цена с НДС, ₽</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="E26" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="F26" s="29" t="n">
+        <v>55200</v>
+      </c>
+      <c r="G26" s="29" t="n">
+        <v>441600</v>
+      </c>
+      <c r="H26" s="29" t="n">
+        <v>79632.78999999999</v>
+      </c>
+      <c r="I26" s="28" t="inlineStr">
+        <is>
+          <t>Ориентир ANDPRO; ~30 суток архива при 51 камере / 3 Мбит/с</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>TRASSIR Neuro Detector — доп. каналы (в 2 NVR уже 4 лицензии)</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>DSSL 26363</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="E27" s="30" t="n">
+        <v>47</v>
+      </c>
+      <c r="F27" s="32" t="n">
+        <v>6600</v>
+      </c>
+      <c r="G27" s="32" t="n">
+        <v>310200</v>
+      </c>
+      <c r="H27" s="32" t="n">
+        <v>55937.7</v>
+      </c>
+      <c r="I27" s="31" t="inlineStr">
+        <is>
+          <t>Опция: аналитика на все 51 камеру</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="33" t="inlineStr">
+        <is>
+          <t>Итого с архивом ~30 суток (позиции 1–6)</t>
+        </is>
+      </c>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="34" t="n"/>
+      <c r="D28" s="34" t="n"/>
+      <c r="E28" s="34" t="n"/>
+      <c r="F28" s="34" t="n"/>
+      <c r="G28" s="35" t="n">
+        <v>2679720</v>
+      </c>
+      <c r="H28" s="35" t="n">
+        <v>483228.2</v>
+      </c>
+      <c r="I28" s="36" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>Итого полный комплект с аналитикой (позиции 1–7)</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="n"/>
+      <c r="C29" s="17" t="n"/>
+      <c r="D29" s="17" t="n"/>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17" t="n"/>
+      <c r="G29" s="18" t="n">
+        <v>2989920</v>
+      </c>
+      <c r="H29" s="18" t="n">
+        <v>539165.9</v>
+      </c>
+      <c r="I29" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>4. Сводка комплектов</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Комплект</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Состав</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Сумма с НДС, ₽</t>
         </is>
       </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>в т.ч. НДС 22%, ₽</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>Примечание</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>HDD 10 ТБ Seagate SkyHawk AI, 3.5" SATA, рекомендован DSSL для NeuroStation 8-disk</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="inlineStr">
-        <is>
-          <t>ST10000VE001</t>
-        </is>
-      </c>
-      <c r="D24" s="27" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-      <c r="E24" s="27" t="n">
-        <v>8</v>
-      </c>
-      <c r="F24" s="29" t="n">
-        <v>55200</v>
-      </c>
-      <c r="G24" s="29" t="n">
-        <v>441600</v>
-      </c>
-      <c r="H24" s="29" t="n">
-        <v>79632.78999999999</v>
-      </c>
-      <c r="I24" s="28" t="inlineStr">
-        <is>
-          <t>Ориентир ANDPRO; ~30 суток архива при 51×4 Мп / 3 Мбит/с</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="30" t="n">
-        <v>5</v>
-      </c>
-      <c r="B25" s="31" t="inlineStr">
-        <is>
-          <t>TRASSIR Neuro Detector — доп. каналы (в 2 NVR уже 4 лицензии)</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr">
-        <is>
-          <t>DSSL 26363</t>
-        </is>
-      </c>
-      <c r="D25" s="30" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-      <c r="E25" s="30" t="n">
-        <v>47</v>
-      </c>
-      <c r="F25" s="32" t="n">
-        <v>6600</v>
-      </c>
-      <c r="G25" s="32" t="n">
-        <v>310200</v>
-      </c>
-      <c r="H25" s="32" t="n">
-        <v>55937.7</v>
-      </c>
-      <c r="I25" s="31" t="inlineStr">
-        <is>
-          <t>Опция: аналитика на все 51 камеру</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="33" t="inlineStr">
-        <is>
-          <t>Итого с архивом ~30 суток (позиции 1–4)</t>
-        </is>
-      </c>
-      <c r="B26" s="34" t="n"/>
-      <c r="C26" s="34" t="n"/>
-      <c r="D26" s="34" t="n"/>
-      <c r="E26" s="34" t="n"/>
-      <c r="F26" s="34" t="n"/>
-      <c r="G26" s="35" t="n">
-        <v>2778670</v>
-      </c>
-      <c r="H26" s="35" t="n">
-        <v>501071.64</v>
-      </c>
-      <c r="I26" s="36" t="n"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>Итого полный комплект с аналитикой (позиции 1–5)</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="n"/>
-      <c r="C27" s="17" t="n"/>
-      <c r="D27" s="17" t="n"/>
-      <c r="E27" s="17" t="n"/>
-      <c r="F27" s="17" t="n"/>
-      <c r="G27" s="18" t="n">
-        <v>3088870</v>
-      </c>
-      <c r="H27" s="18" t="n">
-        <v>557009.34</v>
-      </c>
-      <c r="I27" s="19" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>4. Сводка комплектов</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Комплект</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Состав</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Сумма с НДС, ₽</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>в т.ч. НДС 22%, ₽</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Без НДС, ₽</t>
         </is>
       </c>
-      <c r="F30" s="19" t="n"/>
-      <c r="G30" s="19" t="n"/>
-      <c r="H30" s="19" t="n"/>
-      <c r="I30" s="19" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="37" t="inlineStr">
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="19" t="n"/>
+      <c r="H32" s="19" t="n"/>
+      <c r="I32" s="19" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="37" t="inlineStr">
         <is>
           <t>А. Только запрошенные позиции</t>
         </is>
       </c>
-      <c r="B31" s="38" t="inlineStr">
-        <is>
-          <t>2 NVR + 51 камера</t>
-        </is>
-      </c>
-      <c r="C31" s="39" t="n">
-        <v>2077480</v>
-      </c>
-      <c r="D31" s="39" t="n">
-        <v>374627.54</v>
-      </c>
-      <c r="E31" s="39" t="n">
-        <v>1702852.46</v>
-      </c>
-      <c r="F31" s="40" t="n"/>
-      <c r="G31" s="40" t="n"/>
-      <c r="H31" s="40" t="n"/>
-      <c r="I31" s="40" t="n"/>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="41" t="inlineStr">
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>2 NVR + 1 купол + 49 цилиндр + 1 PTZ</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="n">
+        <v>1978530</v>
+      </c>
+      <c r="D33" s="39" t="n">
+        <v>356784.1</v>
+      </c>
+      <c r="E33" s="39" t="n">
+        <v>1621745.9</v>
+      </c>
+      <c r="F33" s="40" t="n"/>
+      <c r="G33" s="40" t="n"/>
+      <c r="H33" s="40" t="n"/>
+      <c r="I33" s="40" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="41" t="inlineStr">
         <is>
           <t>Б. Работоспособный минимум</t>
         </is>
       </c>
-      <c r="B32" s="42" t="inlineStr">
+      <c r="B34" s="42" t="inlineStr">
         <is>
           <t>А + 51× AnyIP</t>
         </is>
       </c>
-      <c r="C32" s="43" t="n">
-        <v>2337070</v>
-      </c>
-      <c r="D32" s="43" t="n">
-        <v>421438.85</v>
-      </c>
-      <c r="E32" s="43" t="n">
-        <v>1915631.15</v>
-      </c>
-      <c r="F32" s="44" t="n"/>
-      <c r="G32" s="44" t="n"/>
-      <c r="H32" s="44" t="n"/>
-      <c r="I32" s="44" t="n"/>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="45" t="inlineStr">
+      <c r="C34" s="43" t="n">
+        <v>2238120</v>
+      </c>
+      <c r="D34" s="43" t="n">
+        <v>403595.41</v>
+      </c>
+      <c r="E34" s="43" t="n">
+        <v>1834524.59</v>
+      </c>
+      <c r="F34" s="44" t="n"/>
+      <c r="G34" s="44" t="n"/>
+      <c r="H34" s="44" t="n"/>
+      <c r="I34" s="44" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="45" t="inlineStr">
         <is>
           <t>В. С архивом 30 суток</t>
         </is>
       </c>
-      <c r="B33" s="46" t="inlineStr">
+      <c r="B35" s="46" t="inlineStr">
         <is>
           <t>Б + 8× HDD 10 ТБ</t>
         </is>
       </c>
-      <c r="C33" s="47" t="n">
-        <v>2778670</v>
-      </c>
-      <c r="D33" s="47" t="n">
-        <v>501071.64</v>
-      </c>
-      <c r="E33" s="47" t="n">
-        <v>2277598.36</v>
-      </c>
-      <c r="F33" s="48" t="n"/>
-      <c r="G33" s="48" t="n"/>
-      <c r="H33" s="48" t="n"/>
-      <c r="I33" s="48" t="n"/>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="49" t="inlineStr">
+      <c r="C35" s="47" t="n">
+        <v>2679720</v>
+      </c>
+      <c r="D35" s="47" t="n">
+        <v>483228.2</v>
+      </c>
+      <c r="E35" s="47" t="n">
+        <v>2196491.8</v>
+      </c>
+      <c r="F35" s="48" t="n"/>
+      <c r="G35" s="48" t="n"/>
+      <c r="H35" s="48" t="n"/>
+      <c r="I35" s="48" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="49" t="inlineStr">
         <is>
           <t>Г. Полный комплект</t>
         </is>
       </c>
-      <c r="B34" s="50" t="inlineStr">
+      <c r="B36" s="50" t="inlineStr">
         <is>
           <t>В + Neuro Detector на все камеры</t>
         </is>
       </c>
-      <c r="C34" s="51" t="n">
-        <v>3088870</v>
-      </c>
-      <c r="D34" s="51" t="n">
-        <v>557009.34</v>
-      </c>
-      <c r="E34" s="51" t="n">
-        <v>2531860.66</v>
-      </c>
-      <c r="F34" s="52" t="n"/>
-      <c r="G34" s="52" t="n"/>
-      <c r="H34" s="52" t="n"/>
-      <c r="I34" s="52" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="C36" s="51" t="n">
+        <v>2989920</v>
+      </c>
+      <c r="D36" s="51" t="n">
+        <v>539165.9</v>
+      </c>
+      <c r="E36" s="51" t="n">
+        <v>2450754.1</v>
+      </c>
+      <c r="F36" s="52" t="n"/>
+      <c r="G36" s="52" t="n"/>
+      <c r="H36" s="52" t="n"/>
+      <c r="I36" s="52" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>5. Условия и оговорки</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="53" t="inlineStr">
-        <is>
-          <t>• Документ — ориентировочный расчёт по открытым ценам на 14.08.2026, не является офертой. Фиксация — в КП DSSL/дилера TRASSIR и НИЦ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="53" t="inlineStr">
-        <is>
-          <t>• Регистратор поставляется без HDD и без лицензий на подключение IP-камер. В каждом NVR — 2 лицензии Neuro Detector.</t>
-        </is>
-      </c>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="54" t="inlineStr">
-        <is>
-          <t>• Артикул камеры 4BHNN0-0-0-0 в публичных каталогах не найден; по коду — 4 Мп НИЦ «Технологии», прошивка Nexus, базовая комплектация. Корпус и объектив подтвердить до заказа.</t>
+      <c r="A39" s="53" t="inlineStr">
+        <is>
+          <t>• Документ — ориентировочный расчёт по открытым ценам на 14.08.2026, ред. 2. Не оферта. Фиксация — в КП DSSL, НИЦ и ООО «Айпи Плюс».</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="53" t="inlineStr">
-        <is>
-          <t>• Два NVR на 51 камеру: запас каналов 256 vs 51 (резерв, два объекта или расширение). Запись можно вести на одном регистраторе.</t>
+      <c r="A40" s="54" t="inlineStr">
+        <is>
+          <t>• Все камеры поставляются со СТ-1 (и/или номером реестровой записи РЭП). 4MBIR-28-TMLW и 2BPBDD-4794-20: флаг СТ-1 в каталоге IP Plus.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="53" t="inlineStr">
-        <is>
-          <t>• Оценка архива: 51×4 Мп, H.265, 3 Мбит/с ≈ 1,65 ТБ/сутки; 8×10 ТБ достаточно примерно на 30 суток на одном NVR.</t>
+      <c r="A41" s="54" t="inlineStr">
+        <is>
+          <t>• PTZ: взята самая недорогая модель РУВЕР 2 Мп с СТ-1 — 2BPBDD-4794-20 (зум ×20). Модели ×10 в каталоге без СТ-1 не включены.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="53" t="inlineStr">
         <is>
-          <t>• Не включено: PoE-коммутаторы, СКС, шкаф 19", ИБП, мониторы, монтаж, ПНР, доставка.</t>
+          <t>• Регистратор без HDD и без лицензий AnyIP. В каждом NVR — 2 лицензии Neuro Detector.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="53" t="inlineStr">
         <is>
-          <t>• Гарантия TRASSIR — по паспорту (типично 3–5 лет на NVR). Камеры НИЦ — уточняется (часто 3 года).</t>
+          <t>• Оценка архива: 51 камера, H.265, 3 Мбит/с ≈ 1,65 ТБ/сутки; 8×10 ТБ ≈ 30 суток на одном NVR.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="53" t="inlineStr">
         <is>
-          <t>• Контакты: DSSL 8 (800) 100-91-12, dssl.ru, код NVR 80222; НИЦ nic-tech.ru, 8 (800) 555-47-65.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="55" t="inlineStr">
+          <t>• Не включено: PoE-коммутаторы, СКС, шкаф 19", ИБП, мониторы, монтаж, ПНР, доставка.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="53" t="inlineStr">
+        <is>
+          <t>• Контакты: DSSL 8 (800) 100-91-12; НИЦ 8 (800) 555-47-65; Айпи Плюс 8 804 333-73-02, info@ipplus.ru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="55" t="inlineStr">
         <is>
           <t>Поставщик / исполнитель</t>
         </is>
       </c>
-      <c r="F46" s="55" t="inlineStr">
+      <c r="F48" s="55" t="inlineStr">
         <is>
           <t>Заказчик</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>________________ / ________________</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>________________ / ________________</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="56" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="56" t="inlineStr">
         <is>
           <t>подпись, ФИО, дата</t>
         </is>
       </c>
-      <c r="F49" s="56" t="inlineStr">
+      <c r="F51" s="56" t="inlineStr">
         <is>
           <t>подпись, ФИО, дата</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A12:I14"/>
-  <mergeCells count="42">
+  <autoFilter ref="A12:I16"/>
+  <mergeCells count="41">
     <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A37:I37"/>
     <mergeCell ref="C8:I8"/>
-    <mergeCell ref="A27:F27"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="F48:I48"/>
     <mergeCell ref="C7:I7"/>
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F49:I49"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="E35:I35"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A42:I42"/>
     <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="C6:I6"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="E31:I31"/>
-    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A29:F29"/>
     <mergeCell ref="C5:I5"/>
     <mergeCell ref="A38:I38"/>
-    <mergeCell ref="A29:I29"/>
-    <mergeCell ref="E30:I30"/>
     <mergeCell ref="A43:I43"/>
     <mergeCell ref="E34:I34"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="C4:I4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A44:I44"/>
     <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A31:I31"/>
     <mergeCell ref="A39:I39"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="F51:I51"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A24:I24"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F50:I50"/>
     <mergeCell ref="C9:I9"/>
     <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A50:D50"/>
     <mergeCell ref="E32:I32"/>
-    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A45:I45"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="F46:I46"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -1638,7 +1704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1724,100 +1790,140 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="58" t="inlineStr">
         <is>
-          <t>Камера 4 Мп НИЦ (ориентир опта)</t>
+          <t>Купол НИЦ 1143 4MP-DOM-2.7-13.5M Nexus</t>
         </is>
       </c>
       <c r="B6" s="58" t="inlineStr">
         <is>
-          <t>4BHNN0-0-0-0 / NIC-4-BUL-Moto-RUS</t>
+          <t>4MP-DOM-2.7-13.5M</t>
         </is>
       </c>
       <c r="C6" s="59" t="n">
-        <v>22000</v>
+        <v>23800</v>
       </c>
       <c r="D6" s="60" t="inlineStr">
         <is>
-          <t>https://tonzar.com — диапазон 15 000–25 000 ₽, в КП середина 22 000 ₽</t>
+          <t>https://www.nic-tech.ru/upload/iblock/094/ — спецификация модель 1143</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="61" t="inlineStr">
         <is>
-          <t>TRASSIR AnyIP</t>
+          <t>Цилиндр РУВЕР 4 Мп Mini Bullet СТ-1</t>
         </is>
       </c>
       <c r="B7" s="61" t="inlineStr">
         <is>
-          <t>57885</t>
+          <t>4MBIR-28-TMLW</t>
         </is>
       </c>
       <c r="C7" s="63" t="n">
-        <v>5090</v>
+        <v>18500</v>
       </c>
       <c r="D7" s="62" t="inlineStr">
         <is>
-          <t>https://www.dssl.ru/products/trassir-anyip/</t>
+          <t>https://www.ipplus.ru/catalog/ip-kamery/ip-kamery-4mp/4mbir-28-tmlw (цена на сайте не опубликована)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="58" t="inlineStr">
         <is>
-          <t>TRASSIR Neuro Detector</t>
+          <t>PTZ РУВЕР 2 Мп ×20 СТ-1 (самая недорогая с СТ-1)</t>
         </is>
       </c>
       <c r="B8" s="58" t="inlineStr">
         <is>
-          <t>26363</t>
+          <t>2BPBDD-4794-20</t>
         </is>
       </c>
       <c r="C8" s="59" t="n">
-        <v>6600</v>
+        <v>92750</v>
       </c>
       <c r="D8" s="60" t="inlineStr">
         <is>
-          <t>https://www.dssl.ru/products/neuro-detector-nejrosetevoj-detector/</t>
+          <t>https://www.ipplus.ru/catalog/ptz-kamery/ptz-kamery-2mp/2bpbdd-4794-20 ; ориентир класса PTZ20-20x</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="61" t="inlineStr">
         <is>
-          <t>HDD SkyHawk AI 10 ТБ</t>
+          <t>TRASSIR AnyIP</t>
         </is>
       </c>
       <c r="B9" s="61" t="inlineStr">
         <is>
-          <t>ST10000VE001</t>
+          <t>57885</t>
         </is>
       </c>
       <c r="C9" s="63" t="n">
-        <v>55200</v>
+        <v>5090</v>
       </c>
       <c r="D9" s="62" t="inlineStr">
         <is>
-          <t>https://andpro.ru — 55 202 ₽, в КП округлено 55 200 ₽</t>
+          <t>https://www.dssl.ru/products/trassir-anyip/</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="58" t="inlineStr">
         <is>
+          <t>TRASSIR Neuro Detector</t>
+        </is>
+      </c>
+      <c r="B10" s="58" t="inlineStr">
+        <is>
+          <t>26363</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="n">
+        <v>6600</v>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>https://www.dssl.ru/products/neuro-detector-nejrosetevoj-detector/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>HDD SkyHawk AI 10 ТБ</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>ST10000VE001</t>
+        </is>
+      </c>
+      <c r="C11" s="63" t="n">
+        <v>55200</v>
+      </c>
+      <c r="D11" s="62" t="inlineStr">
+        <is>
+          <t>https://andpro.ru — 55 202 ₽, в КП округлено 55 200 ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="58" t="inlineStr">
+        <is>
           <t>Паспорт NVR</t>
         </is>
       </c>
-      <c r="B10" s="58" t="inlineStr">
+      <c r="B12" s="58" t="inlineStr">
         <is>
           <t>Astra 9800R/128-S</t>
         </is>
       </c>
-      <c r="C10" s="58" t="inlineStr">
+      <c r="C12" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D10" s="60" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr">
         <is>
           <t>https://trassir.ru/products/videonablyudenie/videoregistratory/ip_videoregistratory_nvr/trassir_neurostation_98128r_s/</t>
         </is>
@@ -1835,6 +1941,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Recalculate KP on DSSL/TRASSIR camera analogs with ST-1
Replace NIC 1143, RUWARE 4MBIR-28-TMLW and PTZ with TRASSIR ST-1 models TR-D3153IR2 v2 (R), TR-D2151IR3 v2 (R) and TR-D6124IR10 v3 (R). Regenerate Word and Excel as revision 3.

Co-authored-by: Yury1331 <Yury1331@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/kp/2026-08-14-neurostation-4bhnn0/КП_поставка_NeuroStation_Astra_9800R_4BHNN0.xlsx
+++ b/kp/2026-08-14-neurostation-4bhnn0/КП_поставка_NeuroStation_Astra_9800R_4BHNN0.xlsx
@@ -783,7 +783,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>№ КП-2026-08-14-001 ред. 2 от 14.08.2026  ·  2× NVR TRASSIR + 1× НИЦ 1143 + 49× 4MBIR-28-TMLW + 1× PTZ  ·  все камеры со СТ-1  ·  цены с НДС 22%</t>
+          <t>№ КП-2026-08-14-001 ред. 3 от 14.08.2026  ·  2× NVR TRASSIR + 51× камеры TRASSIR СТ-1  ·  1× TR-D3153IR2 + 49× TR-D2151IR3 + 1× PTZ TR-D6124IR10  ·  цены с НДС 22%</t>
         </is>
       </c>
       <c r="B2" s="4" t="n"/>
@@ -830,7 +830,7 @@
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>к заполнению (DSSL / TRASSIR, НИЦ «Технологии», ООО «Айпи Плюс» / РУВЕР)</t>
+          <t>к заполнению (DSSL / авторизованный дилер TRASSIR)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>NVR: 5–15 раб. дней при наличии; камеры НИЦ и РУВЕР — под заказ</t>
+          <t>NVR: 5–15 раб. дней при наличии; камеры СТ-1 — проектная поставка</t>
         </is>
       </c>
     </row>
@@ -978,12 +978,12 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Купольная IP-камера 4 Мп НИЦ модель 1143, мотор 2.7–13.5 мм, ИК до 35 м, IP66/IK10, ПО Nexus. Производство РФ, СТ-1 на партию</t>
+          <t>Аналог НИЦ 1143: уличный вандалостойкий купол TRASSIR 5 Мп, мотор 2.7–13.5 мм, ИК 25 м, IP66/IK10, микрофон. Серия СТ-1 / реестр РЭП</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>4MP-DOM-2.7-13.5M Nexus</t>
+          <t>TR-D3153IR2 v2 (R) 2.7-13.5</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
@@ -995,17 +995,17 @@
         <v>1</v>
       </c>
       <c r="F14" s="15" t="n">
-        <v>23800</v>
+        <v>16380</v>
       </c>
       <c r="G14" s="15" t="n">
-        <v>23800</v>
+        <v>16380</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>4291.8</v>
+        <v>2953.77</v>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>Спецификация НИЦ PDF; ориентир цены 4MP-DOM-2.7-13.5M; СТ-1 запросить на партию</t>
+          <t>DSSL 10100, СТ-1; ориентир цены — розница (D) 16 380 ₽; (R) проектная</t>
         </is>
       </c>
     </row>
@@ -1015,12 +1015,12 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Уличная цилиндрическая IP-камера 4 Мп Mini Bullet, объектив 2.8 мм, ИК + белый свет, микрофон. Производитель РУВЕР, СТ-1</t>
+          <t>Аналог 4MBIR-28-TMLW: уличный цилиндр TRASSIR 5 Мп, фикс 2.8 мм, ИК 35 м, микрофон, IP67. Серия СТ-1 / реестр РЭП</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>4MBIR-28-TMLW</t>
+          <t>TR-D2151IR3 v2 (R) 2.8</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -1032,17 +1032,17 @@
         <v>49</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>18500</v>
+        <v>16800</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>906500</v>
+        <v>823200</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>163467.21</v>
+        <v>148445.9</v>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>https://www.ipplus.ru/catalog/ip-kamery/ip-kamery-4mp/4mbir-28-tmlw ; st_1=true</t>
+          <t>DSSL 16725, СТ-1; ориентир — розница v2 / (D) 16 800 ₽; Dual Light в СТ-1 5 Мп нет</t>
         </is>
       </c>
     </row>
@@ -1052,12 +1052,12 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>PTZ уличная 2 Мп, зум ×20 (4.7–94 мм), IP66. Самая недорогая PTZ РУВЕР/Айпи Плюс с СТ-1 в серии 2 Мп (×10 без СТ-1 не предлагаются)</t>
+          <t>Аналог PTZ: уличная поворотная TRASSIR 2 Мп, зум ×20 (4.3–86 мм), ИК 100 м, IP66/IK10. Самая недорогая PTZ TRASSIR ×20 со СТ-1</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>2BPBDD-4794-20</t>
+          <t>TR-D6124IR10 v3 (R) 4.3-86</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -1069,17 +1069,17 @@
         <v>1</v>
       </c>
       <c r="F16" s="15" t="n">
-        <v>92750</v>
+        <v>49770</v>
       </c>
       <c r="G16" s="15" t="n">
-        <v>92750</v>
+        <v>49770</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>16725.41</v>
+        <v>8974.92</v>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
-          <t>https://www.ipplus.ru/catalog/ptz-kamery/ptz-kamery-2mp/2bpbdd-4794-20 ; реестр Минпромторга</t>
+          <t>DSSL 90684, СТ-1; ориентир — розница v3 / (D) 49 770 ₽</t>
         </is>
       </c>
     </row>
@@ -1095,17 +1095,17 @@
       <c r="E17" s="17" t="n"/>
       <c r="F17" s="17" t="n"/>
       <c r="G17" s="18" t="n">
-        <v>1978530</v>
+        <v>1844830</v>
       </c>
       <c r="H17" s="18" t="n">
-        <v>356784.1</v>
+        <v>332674.26</v>
       </c>
       <c r="I17" s="19" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2. Обязательно к поставке для работоспособности (в регистраторе нет лицензий на IP-камеры; камеры НИЦ/РУВЕР не native TRASSIR)</t>
+          <t>2. Обязательно к поставке для работоспособности (в регистраторе Astra нет лицензий на IP-камеры; AnyIP Astra Linux — DSSL 95887)</t>
         </is>
       </c>
       <c r="B19" s="2" t="n"/>
@@ -1170,12 +1170,12 @@
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>Лицензия TRASSIR AnyIP (TRASSIR OS) — подключение 1 IP-камеры любого производителя</t>
+          <t>Лицензия TRASSIR AnyIP (Astra Linux) — подключение 1 IP-камеры к NeuroStation Astra / UltraStation Astra</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>DSSL 57885</t>
+          <t>DSSL 95887</t>
         </is>
       </c>
       <c r="D21" s="20" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="I21" s="21" t="inlineStr">
         <is>
-          <t>Цена DSSL с 01.04.2026; без лицензии камера к NVR не подключается</t>
+          <t>Для Astra Linux; цена ориентир AnyIP OS 57885. Подарок на камере — уточнить у DSSL</t>
         </is>
       </c>
     </row>
@@ -1213,10 +1213,10 @@
       <c r="E22" s="24" t="n"/>
       <c r="F22" s="24" t="n"/>
       <c r="G22" s="25" t="n">
-        <v>2238120</v>
+        <v>2104420</v>
       </c>
       <c r="H22" s="25" t="n">
-        <v>403595.41</v>
+        <v>379485.57</v>
       </c>
       <c r="I22" s="26" t="n"/>
     </row>
@@ -1368,10 +1368,10 @@
       <c r="E28" s="34" t="n"/>
       <c r="F28" s="34" t="n"/>
       <c r="G28" s="35" t="n">
-        <v>2679720</v>
+        <v>2546020</v>
       </c>
       <c r="H28" s="35" t="n">
-        <v>483228.2</v>
+        <v>459118.36</v>
       </c>
       <c r="I28" s="36" t="n"/>
     </row>
@@ -1387,10 +1387,10 @@
       <c r="E29" s="17" t="n"/>
       <c r="F29" s="17" t="n"/>
       <c r="G29" s="18" t="n">
-        <v>2989920</v>
+        <v>2856220</v>
       </c>
       <c r="H29" s="18" t="n">
-        <v>539165.9</v>
+        <v>515056.07</v>
       </c>
       <c r="I29" s="19" t="n"/>
     </row>
@@ -1448,17 +1448,17 @@
       </c>
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>2 NVR + 1 купол + 49 цилиндр + 1 PTZ</t>
+          <t>2 NVR + 1 купол + 49 цилиндр + 1 PTZ TRASSIR</t>
         </is>
       </c>
       <c r="C33" s="39" t="n">
-        <v>1978530</v>
+        <v>1844830</v>
       </c>
       <c r="D33" s="39" t="n">
-        <v>356784.1</v>
+        <v>332674.26</v>
       </c>
       <c r="E33" s="39" t="n">
-        <v>1621745.9</v>
+        <v>1512155.74</v>
       </c>
       <c r="F33" s="40" t="n"/>
       <c r="G33" s="40" t="n"/>
@@ -1477,13 +1477,13 @@
         </is>
       </c>
       <c r="C34" s="43" t="n">
-        <v>2238120</v>
+        <v>2104420</v>
       </c>
       <c r="D34" s="43" t="n">
-        <v>403595.41</v>
+        <v>379485.57</v>
       </c>
       <c r="E34" s="43" t="n">
-        <v>1834524.59</v>
+        <v>1724934.43</v>
       </c>
       <c r="F34" s="44" t="n"/>
       <c r="G34" s="44" t="n"/>
@@ -1502,13 +1502,13 @@
         </is>
       </c>
       <c r="C35" s="47" t="n">
-        <v>2679720</v>
+        <v>2546020</v>
       </c>
       <c r="D35" s="47" t="n">
-        <v>483228.2</v>
+        <v>459118.36</v>
       </c>
       <c r="E35" s="47" t="n">
-        <v>2196491.8</v>
+        <v>2086901.64</v>
       </c>
       <c r="F35" s="48" t="n"/>
       <c r="G35" s="48" t="n"/>
@@ -1527,13 +1527,13 @@
         </is>
       </c>
       <c r="C36" s="51" t="n">
-        <v>2989920</v>
+        <v>2856220</v>
       </c>
       <c r="D36" s="51" t="n">
-        <v>539165.9</v>
+        <v>515056.07</v>
       </c>
       <c r="E36" s="51" t="n">
-        <v>2450754.1</v>
+        <v>2341163.93</v>
       </c>
       <c r="F36" s="52" t="n"/>
       <c r="G36" s="52" t="n"/>
@@ -1558,49 +1558,56 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="53" t="inlineStr">
         <is>
-          <t>• Документ — ориентировочный расчёт по открытым ценам на 14.08.2026, ред. 2. Не оферта. Фиксация — в КП DSSL, НИЦ и ООО «Айпи Плюс».</t>
+          <t>• Документ — ориентировочный расчёт по открытым ценам на 14.08.2026, ред. 3. Не оферта. Фиксация — в КП DSSL / дилера TRASSIR.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="54" t="inlineStr">
         <is>
-          <t>• Все камеры поставляются со СТ-1 (и/или номером реестровой записи РЭП). 4MBIR-28-TMLW и 2BPBDD-4794-20: флаг СТ-1 в каталоге IP Plus.</t>
+          <t>• Всё оборудование — DSSL/TRASSIR. Камеры — исполнения (R) со СТ-1 и записью в РЭП (ПП РФ №878).</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="54" t="inlineStr">
         <is>
-          <t>• PTZ: взята самая недорогая модель РУВЕР 2 Мп с СТ-1 — 2BPBDD-4794-20 (зум ×20). Модели ×10 в каталоге без СТ-1 не включены.</t>
+          <t>• Подбор: НИЦ 1143 → TR-D3153IR2 v2 (R); 4MBIR-28-TMLW → TR-D2151IR3 v2 (R); PTZ → TR-D6124IR10 v3 (R) ×20.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="53" t="inlineStr">
         <is>
-          <t>• Регистратор без HDD и без лицензий AnyIP. В каждом NVR — 2 лицензии Neuro Detector.</t>
+          <t>• В линейке СТ-1 нет 4 Мп: взяты ближайшие 5 Мп. Dual Light (ИК+белый) в СТ-1 5 Мп нет — у цилиндра только ИК.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="53" t="inlineStr">
         <is>
-          <t>• Оценка архива: 51 камера, H.265, 3 Мбит/с ≈ 1,65 ТБ/сутки; 8×10 ТБ ≈ 30 суток на одном NVR.</t>
+          <t>• Регистратор без HDD. Лицензии AnyIP (Astra Linux, 95887) в NVR нет; «ПО в подарок» на камере — уточнить для Astra.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="53" t="inlineStr">
         <is>
-          <t>• Не включено: PoE-коммутаторы, СКС, шкаф 19", ИБП, мониторы, монтаж, ПНР, доставка.</t>
+          <t>• Оценка архива: 51 камера, H.265, 3 Мбит/с ≈ 1,65 ТБ/сутки; 8×10 ТБ ≈ 30 суток на одном NVR.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="53" t="inlineStr">
         <is>
-          <t>• Контакты: DSSL 8 (800) 100-91-12; НИЦ 8 (800) 555-47-65; Айпи Плюс 8 804 333-73-02, info@ipplus.ru.</t>
+          <t>• Не включено: PoE-коммутаторы, СКС, шкаф 19", ИБП, мониторы, монтаж, ПНР, доставка.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="53" t="inlineStr">
+        <is>
+          <t>• Контакты: DSSL 8 (800) 100-91-12, dssl.ru; коды: NVR 80222, купол 10100, цилиндр 16725, PTZ 90684, AnyIP Astra 95887.</t>
         </is>
       </c>
     </row>
@@ -1642,8 +1649,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A12:I16"/>
-  <mergeCells count="41">
+  <mergeCells count="42">
     <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A46:I46"/>
     <mergeCell ref="C8:I8"/>
     <mergeCell ref="E33:I33"/>
     <mergeCell ref="F48:I48"/>
@@ -1790,72 +1798,72 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="58" t="inlineStr">
         <is>
-          <t>Купол НИЦ 1143 4MP-DOM-2.7-13.5M Nexus</t>
+          <t>Купол TRASSIR СТ-1 5 Мп мотор 2.7–13.5 (аналог 1143)</t>
         </is>
       </c>
       <c r="B6" s="58" t="inlineStr">
         <is>
-          <t>4MP-DOM-2.7-13.5M</t>
+          <t>TR-D3153IR2 v2 (R) 2.7-13.5</t>
         </is>
       </c>
       <c r="C6" s="59" t="n">
-        <v>23800</v>
+        <v>16380</v>
       </c>
       <c r="D6" s="60" t="inlineStr">
         <is>
-          <t>https://www.nic-tech.ru/upload/iblock/094/ — спецификация модель 1143</t>
+          <t>https://www.dssl.ru/products/tr-d3153ir2-v2-r-2-7-13-5-ip-kamera/ — ориентир (D) 16 380 ₽</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="61" t="inlineStr">
         <is>
-          <t>Цилиндр РУВЕР 4 Мп Mini Bullet СТ-1</t>
+          <t>Цилиндр TRASSIR СТ-1 5 Мп 2.8 мм (аналог 4MBIR)</t>
         </is>
       </c>
       <c r="B7" s="61" t="inlineStr">
         <is>
-          <t>4MBIR-28-TMLW</t>
+          <t>TR-D2151IR3 v2 (R) 2.8</t>
         </is>
       </c>
       <c r="C7" s="63" t="n">
-        <v>18500</v>
+        <v>16800</v>
       </c>
       <c r="D7" s="62" t="inlineStr">
         <is>
-          <t>https://www.ipplus.ru/catalog/ip-kamery/ip-kamery-4mp/4mbir-28-tmlw (цена на сайте не опубликована)</t>
+          <t>https://www.dssl.ru/products/tr-d2151ir3-v2-r-2-8-ip-kamera/ — ориентир v2 16 800 ₽</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="58" t="inlineStr">
         <is>
-          <t>PTZ РУВЕР 2 Мп ×20 СТ-1 (самая недорогая с СТ-1)</t>
+          <t>PTZ TRASSIR СТ-1 2 Мп ×20 (самая недорогая ×20)</t>
         </is>
       </c>
       <c r="B8" s="58" t="inlineStr">
         <is>
-          <t>2BPBDD-4794-20</t>
+          <t>TR-D6124IR10 v3 (R) 4.3-86</t>
         </is>
       </c>
       <c r="C8" s="59" t="n">
-        <v>92750</v>
+        <v>49770</v>
       </c>
       <c r="D8" s="60" t="inlineStr">
         <is>
-          <t>https://www.ipplus.ru/catalog/ptz-kamery/ptz-kamery-2mp/2bpbdd-4794-20 ; ориентир класса PTZ20-20x</t>
+          <t>https://www.dssl.ru/products/tr-d6124ir10-v3-r-4-3-86-ip-kamera/ — ориентир v3 49 770 ₽</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="61" t="inlineStr">
         <is>
-          <t>TRASSIR AnyIP</t>
+          <t>TRASSIR AnyIP (Astra Linux)</t>
         </is>
       </c>
       <c r="B9" s="61" t="inlineStr">
         <is>
-          <t>57885</t>
+          <t>95887</t>
         </is>
       </c>
       <c r="C9" s="63" t="n">
@@ -1863,7 +1871,7 @@
       </c>
       <c r="D9" s="62" t="inlineStr">
         <is>
-          <t>https://www.dssl.ru/products/trassir-anyip/</t>
+          <t>https://www.dssl.ru/products/litsenziya-trassir-anyip-astra-linux/ (проектная; ориентир AnyIP OS 57885)</t>
         </is>
       </c>
     </row>

</xml_diff>